<commit_message>
📅 fix: Quote dotted date formats safely and apply them to the preview
The dot-quoting regex rewrote every `.` in the number format, including
dots inside `"..."` literals and after a backslash escape. A format such as
`d. mmmm yyyy "kl." hh:mm` became unbalanced, SheetJS still threw, and the
cell stayed a serial. Skip quoted runs and escaped characters so only bare
separator dots are quoted.

The rich spreadsheet preview reads the workbook on its own path and never
ran the date fill, so the same cell showed a serial in the preview and a
date in the chat text. Move the helper to `spreadsheetDates.ts` as a
workbook-level function and call it from both `excelSheetToText` and
`excelSheetToHtml`.

Extend the fixture with a quoted-literal format, a backslash-escaped format
and a fractional-seconds format, and cover the preview path in html.spec.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packages/api/src/files/documents/sample-dotted-dates.xlsx
+++ b/packages/api/src/files/documents/sample-dotted-dates.xlsx
@@ -1,40 +1,59 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Dates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dates" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="dd.mm.yyyy"/>
-    <numFmt numFmtId="166" formatCode="dd.mm"/>
-    <numFmt numFmtId="167" formatCode="d.m.yyyy"/>
-    <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="8">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="60" formatCode="dd.mm.yyyy"/>
+    <numFmt numFmtId="61" formatCode="dd.mm"/>
+    <numFmt numFmtId="62" formatCode="d.m.yyyy"/>
+    <numFmt numFmtId="63" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="64" formatCode="d. mmmm yyyy &quot;kl.&quot; hh:mm"/>
+    <numFmt numFmtId="65" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="66" formatCode="hh:mm:ss.0"/>
   </numFmts>
   <fonts count="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -52,86 +71,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="9">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="61" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="62" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="63" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="64" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="65" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="66" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
@@ -210,6 +165,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -244,6 +200,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -278,20 +235,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -413,83 +366,129 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B9"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Format</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+      <c r="A1" t="str">
+        <v>Format</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Value</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>dd.mm.yyyy</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="n">
+      <c r="A2" t="str">
+        <v>dd.mm.yyyy</v>
+      </c>
+      <c r="B2" s="1">
         <v>46265</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>dd.mm</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
+      <c r="A3" t="str">
+        <v>dd.mm</v>
+      </c>
+      <c r="B3" s="2">
         <v>46266</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>d.m.yyyy</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
+      <c r="A4" t="str">
+        <v>d.m.yyyy</v>
+      </c>
+      <c r="B4" s="3">
         <v>46241</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>dd/mm/yyyy</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
+      <c r="A5" t="str">
+        <v>dd/mm/yyyy</v>
+      </c>
+      <c r="B5" s="4">
         <v>46265</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>#,##0.00</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
+      <c r="A6" t="str">
+        <v>#,##0.00</v>
+      </c>
+      <c r="B6" s="5">
         <v>1234.5</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>d. mmmm yyyy "kl." hh:mm</v>
+      </c>
+      <c r="B7" s="6">
+        <v>46265.52431</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>dd\.mm\.yyyy</v>
+      </c>
+      <c r="B8" s="7">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>hh:mm:ss.0</v>
+      </c>
+      <c r="B9" s="8">
+        <v>46265.52431</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>